<commit_message>
Auto commit: 2026-06-04 17:18
</commit_message>
<xml_diff>
--- a/data/metadata/lqas_metadata.xlsx
+++ b/data/metadata/lqas_metadata.xlsx
@@ -423,7 +423,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-05-19 16:50:22</t>
+          <t>2026-06-04 09:40:42</t>
         </is>
       </c>
     </row>
@@ -8837,7 +8837,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-05-19 16:50:22</t>
+          <t>2026-06-04 09:40:42</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto commit: 2026-06-10 16:30
</commit_message>
<xml_diff>
--- a/data/metadata/lqas_metadata.xlsx
+++ b/data/metadata/lqas_metadata.xlsx
@@ -423,7 +423,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-06-04 09:40:42</t>
+          <t>2026-06-10 09:54:28</t>
         </is>
       </c>
     </row>
@@ -8837,7 +8837,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-06-04 09:40:42</t>
+          <t>2026-06-10 09:54:28</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto commit: 2026-06-11 16:32
</commit_message>
<xml_diff>
--- a/data/metadata/lqas_metadata.xlsx
+++ b/data/metadata/lqas_metadata.xlsx
@@ -423,7 +423,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-06-10 09:54:28</t>
+          <t>2026-06-11 13:06:20</t>
         </is>
       </c>
     </row>
@@ -8837,7 +8837,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-06-10 09:54:28</t>
+          <t>2026-06-11 13:06:20</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto commit: 2026-06-17 16:30
</commit_message>
<xml_diff>
--- a/data/metadata/lqas_metadata.xlsx
+++ b/data/metadata/lqas_metadata.xlsx
@@ -423,7 +423,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-06-11 13:06:20</t>
+          <t>2026-06-17 10:04:19</t>
         </is>
       </c>
     </row>
@@ -8837,7 +8837,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-06-11 13:06:20</t>
+          <t>2026-06-17 10:04:19</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto commit: 2026-08-18 07:55
</commit_message>
<xml_diff>
--- a/data/metadata/lqas_metadata.xlsx
+++ b/data/metadata/lqas_metadata.xlsx
@@ -423,7 +423,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-08-15 16:32:42</t>
+          <t>2026-08-17 11:24:05</t>
         </is>
       </c>
     </row>
@@ -8622,7 +8622,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-08-15 16:32:42</t>
+          <t>2026-08-17 11:24:05</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto commit: 2026-08-19 12:29
</commit_message>
<xml_diff>
--- a/data/metadata/lqas_metadata.xlsx
+++ b/data/metadata/lqas_metadata.xlsx
@@ -423,7 +423,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-08-17 11:24:05</t>
+          <t>2026-08-18 12:54:05</t>
         </is>
       </c>
     </row>
@@ -8622,7 +8622,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-08-17 11:24:05</t>
+          <t>2026-08-18 12:54:05</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto commit: 2026-08-27 08:02
</commit_message>
<xml_diff>
--- a/data/metadata/lqas_metadata.xlsx
+++ b/data/metadata/lqas_metadata.xlsx
@@ -423,7 +423,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-08-18 12:54:05</t>
+          <t>2026-08-25 13:54:24</t>
         </is>
       </c>
     </row>
@@ -8622,7 +8622,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-08-18 12:54:05</t>
+          <t>2026-08-25 13:54:24</t>
         </is>
       </c>
     </row>

</xml_diff>